<commit_message>
docs: remove old YAML refs from design spec
- Remove yaml_examples block (protocol_example, commands_example, telemetry_example)
- Remove protocol_template.xlsx reference
- Fix config_templates description (remove '和 YAML 模板参考')
- Update scripts section to use actual script names
</commit_message>
<xml_diff>
--- a/项目文档/excel版遥测大表草稿/固定地址参数注入1.xlsx
+++ b/项目文档/excel版遥测大表草稿/固定地址参数注入1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Codex Workspace\02_Projects\项目文档\excel版遥测大表\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Codex Workspace\04_projects\项目文档\excel版遥测大表草稿\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E051FE2-FFCF-4720-8A43-9FE5E661746F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE6C3F3F-7411-48C8-BE44-0633DD54D1D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="160">
   <si>
     <t>序号</t>
   </si>
@@ -44,22 +44,6 @@
   </si>
   <si>
     <t>参数名称</t>
-  </si>
-  <si>
-    <t>数据域偏移
-data_offset</t>
-  </si>
-  <si>
-    <t>位偏移
-bit_offset</t>
-  </si>
-  <si>
-    <t>位长度
-bit_length</t>
-  </si>
-  <si>
-    <t>数据类型
-type</t>
   </si>
   <si>
     <t>TCT4001</t>
@@ -399,10 +383,6 @@
     <t>标识符</t>
   </si>
   <si>
-    <t>参数值</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>float</t>
   </si>
   <si>
@@ -413,31 +393,12 @@
   </si>
   <si>
     <t>压传IIR滤波器系数a5</t>
-  </si>
-  <si>
-    <t>字节序
-endian</t>
-  </si>
-  <si>
-    <t>小数位数
-decimal_places</t>
-  </si>
-  <si>
-    <t>单位
-unit</t>
-  </si>
-  <si>
-    <t>big</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>指令码</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>层级</t>
-  </si>
-  <si>
     <t>区域</t>
   </si>
   <si>
@@ -450,22 +411,7 @@
     <t>说明</t>
   </si>
   <si>
-    <t>数据包</t>
-  </si>
-  <si>
     <t>包主导头</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>0xEB90</t>
-  </si>
-  <si>
-    <t>版本+类型+副导头+APID</t>
-  </si>
-  <si>
-    <t>0x0520</t>
   </si>
   <si>
     <t>数据域长度</t>
@@ -496,14 +442,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>源包序列号</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0b11</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>0x00~0x3FFF</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -516,15 +454,149 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>初始值</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>取值范围</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>0x03FF</t>
+    <t>参数值(十进制)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+      </rPr>
+      <t>转换方式</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>高字节在前，浮点数IEEE754格式</t>
+  </si>
+  <si>
+    <t>高字节在前，浮点数IEEE754格式</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>值类型</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>数值参数</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>APID</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>源包序列计数</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>位偏移</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>参数1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>参数2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>初始值(HEX)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>EB90</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0520</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>11</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>03FF</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>big_endian</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">位长度
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>bit_length</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">位偏移
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>bit_offset</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>数据类型</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>字节序</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>小数位数</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>单位</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -532,7 +604,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -577,6 +649,21 @@
       <family val="2"/>
       <charset val="134"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="等线"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -597,7 +684,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -650,11 +737,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -670,6 +768,22 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -952,13 +1066,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="28.08203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="28.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="58" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="31" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -969,46 +1084,48 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>137</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="I1" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="J1" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="K1" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="D2" s="3">
         <v>240</v>
       </c>
-      <c r="E2">
-        <f>INT(F2/8)-8</f>
-        <v>2</v>
+      <c r="E2" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F2">
         <v>80</v>
@@ -1017,31 +1134,33 @@
         <v>32</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I2" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J2">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D3" s="3">
         <v>120</v>
       </c>
-      <c r="E3">
-        <f t="shared" ref="E3:E58" si="0">INT(F3/8)-8</f>
-        <v>6</v>
+      <c r="E3" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F3">
         <f>F2+G2</f>
@@ -1051,1883 +1170,1996 @@
         <v>32</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I3" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J3">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L3" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D4" s="3">
         <v>300</v>
       </c>
-      <c r="E4">
-        <f t="shared" si="0"/>
-        <v>10</v>
+      <c r="E4" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F4">
-        <f t="shared" ref="F4:F58" si="1">F3+G3</f>
+        <f t="shared" ref="F4:F58" si="0">F3+G3</f>
         <v>144</v>
       </c>
       <c r="G4">
         <v>32</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I4" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J4">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L4" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D5" s="3">
         <v>300</v>
       </c>
-      <c r="E5">
-        <f t="shared" si="0"/>
-        <v>14</v>
+      <c r="E5" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F5">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>176</v>
       </c>
       <c r="G5">
         <v>32</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="I5" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J5">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L5" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D6" s="3">
         <v>360</v>
       </c>
-      <c r="E6">
-        <f t="shared" si="0"/>
-        <v>18</v>
+      <c r="E6" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>208</v>
       </c>
       <c r="G6">
         <v>32</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I6" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J6">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L6" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D7" s="3">
         <v>10</v>
       </c>
-      <c r="E7">
-        <f t="shared" si="0"/>
-        <v>22</v>
+      <c r="E7" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>240</v>
       </c>
       <c r="G7">
         <v>32</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I7" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J7">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L7" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D8" s="3">
         <v>3000</v>
       </c>
-      <c r="E8">
-        <f t="shared" si="0"/>
-        <v>26</v>
+      <c r="E8" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>272</v>
       </c>
       <c r="G8">
         <v>32</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I8" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J8">
         <v>3</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L8" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D9" s="3">
         <v>1800</v>
       </c>
-      <c r="E9">
-        <f t="shared" si="0"/>
-        <v>30</v>
+      <c r="E9" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>304</v>
       </c>
       <c r="G9">
         <v>32</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I9" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J9">
         <v>3</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L9" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D10" s="3">
         <v>1800</v>
       </c>
-      <c r="E10">
-        <f t="shared" si="0"/>
-        <v>34</v>
+      <c r="E10" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>336</v>
       </c>
       <c r="G10">
         <v>32</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I10" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J10">
         <v>3</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L10" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D11" s="3">
         <v>5400</v>
       </c>
-      <c r="E11">
-        <f t="shared" si="0"/>
-        <v>38</v>
+      <c r="E11" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>368</v>
       </c>
       <c r="G11">
         <v>32</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I11" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J11">
         <v>3</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L11" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D12" s="3">
         <v>600</v>
       </c>
-      <c r="E12">
-        <f t="shared" si="0"/>
-        <v>42</v>
+      <c r="E12" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>400</v>
       </c>
       <c r="G12">
         <v>32</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I12" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J12">
         <v>3</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L12" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D13" s="3">
         <v>300</v>
       </c>
-      <c r="E13">
-        <f t="shared" si="0"/>
-        <v>46</v>
+      <c r="E13" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>432</v>
       </c>
       <c r="G13">
         <v>32</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I13" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J13">
         <v>3</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L13" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D14" s="3">
         <v>600</v>
       </c>
-      <c r="E14">
-        <f t="shared" si="0"/>
-        <v>50</v>
+      <c r="E14" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>464</v>
       </c>
       <c r="G14">
         <v>32</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I14" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J14">
         <v>3</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L14" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D15" s="3">
         <v>60</v>
       </c>
-      <c r="E15">
-        <f t="shared" si="0"/>
-        <v>54</v>
+      <c r="E15" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F15">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>496</v>
       </c>
       <c r="G15">
         <v>32</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I15" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J15">
         <v>3</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L15" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D16" s="3">
         <v>5</v>
       </c>
-      <c r="E16">
-        <f t="shared" si="0"/>
-        <v>58</v>
+      <c r="E16" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>528</v>
       </c>
       <c r="G16">
         <v>32</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I16" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J16">
         <v>3</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="L16" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D17" s="3">
         <v>60</v>
       </c>
-      <c r="E17">
-        <f t="shared" si="0"/>
-        <v>62</v>
+      <c r="E17" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>560</v>
       </c>
       <c r="G17">
         <v>32</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I17" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J17">
         <v>3</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="L17" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D18" s="3">
         <v>50</v>
       </c>
-      <c r="E18">
-        <f t="shared" si="0"/>
-        <v>66</v>
+      <c r="E18" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>592</v>
       </c>
       <c r="G18">
         <v>32</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I18" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J18">
         <v>3</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="L18" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D19" s="3">
         <v>30</v>
       </c>
-      <c r="E19">
-        <f t="shared" si="0"/>
-        <v>70</v>
+      <c r="E19" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>624</v>
       </c>
       <c r="G19">
         <v>32</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="I19" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J19">
         <v>3</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="L19" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D20" s="3">
         <v>2</v>
       </c>
-      <c r="E20">
-        <f t="shared" si="0"/>
-        <v>74</v>
+      <c r="E20" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>656</v>
       </c>
       <c r="G20">
         <v>32</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="I20" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J20">
         <v>3</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="L20" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D21" s="3">
         <v>60</v>
       </c>
-      <c r="E21">
-        <f t="shared" si="0"/>
-        <v>78</v>
+      <c r="E21" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F21">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>688</v>
       </c>
       <c r="G21">
         <v>32</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I21" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J21">
         <v>3</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="L21" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D22" s="3">
         <v>0.5</v>
       </c>
-      <c r="E22">
-        <f t="shared" si="0"/>
-        <v>82</v>
+      <c r="E22" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>720</v>
       </c>
       <c r="G22">
         <v>32</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I22" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J22">
         <v>3</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="L22" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D23" s="3">
         <v>3.15E-2</v>
       </c>
-      <c r="E23">
-        <f t="shared" si="0"/>
-        <v>86</v>
+      <c r="E23" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>752</v>
       </c>
       <c r="G23">
         <v>32</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I23" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J23">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="L23" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D24" s="3">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="E24">
-        <f t="shared" si="0"/>
-        <v>90</v>
+      <c r="E24" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F24">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>784</v>
       </c>
       <c r="G24">
         <v>32</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I24" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J24">
         <v>3</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="L24" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D25" s="3">
         <v>2E-3</v>
       </c>
-      <c r="E25">
-        <f t="shared" si="0"/>
-        <v>94</v>
+      <c r="E25" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F25">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>816</v>
       </c>
       <c r="G25">
         <v>32</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I25" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J25">
         <v>3</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="L25" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D26" s="3">
         <v>3</v>
       </c>
-      <c r="E26">
-        <f t="shared" si="0"/>
-        <v>98</v>
+      <c r="E26" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>848</v>
       </c>
       <c r="G26">
         <v>32</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I26" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J26">
         <v>3</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="L26" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D27" s="3">
         <v>1</v>
       </c>
-      <c r="E27">
-        <f t="shared" si="0"/>
-        <v>102</v>
+      <c r="E27" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>880</v>
       </c>
       <c r="G27">
         <v>32</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I27" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J27">
         <v>3</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="L27" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D28" s="3">
         <v>0.2</v>
       </c>
-      <c r="E28">
-        <f t="shared" si="0"/>
-        <v>106</v>
+      <c r="E28" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>912</v>
       </c>
       <c r="G28">
         <v>32</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I28" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J28">
         <v>3</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="L28" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D29" s="3">
         <v>0.02</v>
       </c>
-      <c r="E29">
-        <f t="shared" si="0"/>
-        <v>110</v>
+      <c r="E29" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>944</v>
       </c>
       <c r="G29">
         <v>32</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I29" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J29">
         <v>3</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="L29" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D30" s="3">
         <v>0.2</v>
       </c>
-      <c r="E30">
-        <f t="shared" si="0"/>
-        <v>114</v>
+      <c r="E30" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F30">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>976</v>
       </c>
       <c r="G30">
         <v>32</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I30" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J30">
         <v>3</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="L30" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D31" s="3">
         <v>2</v>
       </c>
-      <c r="E31">
-        <f t="shared" si="0"/>
-        <v>118</v>
+      <c r="E31" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F31">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1008</v>
       </c>
       <c r="G31">
         <v>32</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="I31" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J31">
         <v>3</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="L31" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D32" s="3">
         <v>-1.2200000000000001E-2</v>
       </c>
-      <c r="E32">
-        <f t="shared" si="0"/>
-        <v>122</v>
+      <c r="E32" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1040</v>
       </c>
       <c r="G32">
         <v>32</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I32" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J32">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L32" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D33" s="3">
         <v>-2.1014000000000001E-2</v>
       </c>
-      <c r="E33">
-        <f t="shared" si="0"/>
-        <v>126</v>
+      <c r="E33" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F33">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1072</v>
       </c>
       <c r="G33">
         <v>32</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I33" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J33">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L33" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D34" s="3">
         <v>-2.4590999999999998E-2</v>
       </c>
-      <c r="E34">
-        <f t="shared" si="0"/>
-        <v>130</v>
+      <c r="E34" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F34">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1104</v>
       </c>
       <c r="G34">
         <v>32</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I34" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J34">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L34" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D35" s="3">
         <v>-1.1148E-2</v>
       </c>
-      <c r="E35">
-        <f t="shared" si="0"/>
-        <v>134</v>
+      <c r="E35" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F35">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1136</v>
       </c>
       <c r="G35">
         <v>32</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I35" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J35">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L35" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D36" s="3">
         <v>2.5974000000000001E-2</v>
       </c>
-      <c r="E36">
-        <f t="shared" si="0"/>
-        <v>138</v>
+      <c r="E36" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1168</v>
       </c>
       <c r="G36">
         <v>32</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I36" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J36">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L36" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D37" s="3">
         <v>8.3951999999999999E-2</v>
       </c>
-      <c r="E37">
-        <f t="shared" si="0"/>
+      <c r="E37" s="8" t="s">
         <v>142</v>
       </c>
       <c r="F37">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1200</v>
       </c>
       <c r="G37">
         <v>32</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I37" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J37">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L37" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D38" s="3">
         <v>0.14888799999999999</v>
       </c>
-      <c r="E38">
-        <f t="shared" si="0"/>
-        <v>146</v>
+      <c r="E38" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1232</v>
       </c>
       <c r="G38">
         <v>32</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I38" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J38">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L38" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D39" s="3">
         <v>0.20025299999999999</v>
       </c>
-      <c r="E39">
-        <f t="shared" si="0"/>
-        <v>150</v>
+      <c r="E39" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1264</v>
       </c>
       <c r="G39">
         <v>32</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I39" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J39">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L39" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D40" s="3">
         <v>0.219802</v>
       </c>
-      <c r="E40">
-        <f t="shared" si="0"/>
-        <v>154</v>
+      <c r="E40" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F40">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1296</v>
       </c>
       <c r="G40">
         <v>32</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I40" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J40">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L40" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D41" s="3">
         <v>-1.2200000000000001E-2</v>
       </c>
-      <c r="E41">
-        <f t="shared" si="0"/>
-        <v>158</v>
+      <c r="E41" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1328</v>
       </c>
       <c r="G41">
         <v>32</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I41" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J41">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L41" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D42" s="3">
         <v>-2.1014000000000001E-2</v>
       </c>
-      <c r="E42">
-        <f t="shared" si="0"/>
-        <v>162</v>
+      <c r="E42" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F42">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1360</v>
       </c>
       <c r="G42">
         <v>32</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I42" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J42">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L42" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D43" s="3">
         <v>-2.4590999999999998E-2</v>
       </c>
-      <c r="E43">
-        <f t="shared" si="0"/>
-        <v>166</v>
+      <c r="E43" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F43">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1392</v>
       </c>
       <c r="G43">
         <v>32</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I43" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J43">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L43" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D44" s="3">
         <v>-1.1148E-2</v>
       </c>
-      <c r="E44">
-        <f t="shared" si="0"/>
-        <v>170</v>
+      <c r="E44" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1424</v>
       </c>
       <c r="G44">
         <v>32</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I44" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J44">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L44" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="D45" s="3">
         <v>2.5974000000000001E-2</v>
       </c>
-      <c r="E45">
-        <f t="shared" si="0"/>
-        <v>174</v>
+      <c r="E45" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F45">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1456</v>
       </c>
       <c r="G45">
         <v>32</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I45" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J45">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L45" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="D46" s="3">
         <v>8.3951999999999999E-2</v>
       </c>
-      <c r="E46">
-        <f t="shared" si="0"/>
-        <v>178</v>
+      <c r="E46" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1488</v>
       </c>
       <c r="G46">
         <v>32</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I46" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J46">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L46" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="D47" s="3">
         <v>0.14888799999999999</v>
       </c>
-      <c r="E47">
-        <f t="shared" si="0"/>
-        <v>182</v>
+      <c r="E47" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F47">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1520</v>
       </c>
       <c r="G47">
         <v>32</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I47" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J47">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L47" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D48" s="3">
         <v>0.20025299999999999</v>
       </c>
-      <c r="E48">
-        <f t="shared" si="0"/>
-        <v>186</v>
+      <c r="E48" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F48">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1552</v>
       </c>
       <c r="G48">
         <v>32</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I48" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J48">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L48" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D49" s="3">
         <v>0.219802</v>
       </c>
-      <c r="E49">
-        <f t="shared" si="0"/>
-        <v>190</v>
+      <c r="E49" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F49">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1584</v>
       </c>
       <c r="G49">
         <v>32</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I49" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J49">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L49" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D50" s="3">
         <v>-1.2200000000000001E-2</v>
       </c>
-      <c r="E50">
-        <f t="shared" si="0"/>
-        <v>194</v>
+      <c r="E50" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F50">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1616</v>
       </c>
       <c r="G50">
         <v>32</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I50" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J50">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L50" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D51" s="3">
         <v>-2.1014000000000001E-2</v>
       </c>
-      <c r="E51">
-        <f t="shared" si="0"/>
-        <v>198</v>
+      <c r="E51" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F51">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1648</v>
       </c>
       <c r="G51">
         <v>32</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I51" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J51">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L51" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D52" s="3">
         <v>-2.4590999999999998E-2</v>
       </c>
-      <c r="E52">
-        <f t="shared" si="0"/>
-        <v>202</v>
+      <c r="E52" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F52">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1680</v>
       </c>
       <c r="G52">
         <v>32</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I52" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J52">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L52" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D53" s="3">
         <v>-1.1148E-2</v>
       </c>
-      <c r="E53">
-        <f t="shared" si="0"/>
-        <v>206</v>
+      <c r="E53" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F53">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1712</v>
       </c>
       <c r="G53">
         <v>32</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I53" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J53">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L53" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D54" s="3">
         <v>2.5974000000000001E-2</v>
       </c>
-      <c r="E54">
-        <f t="shared" si="0"/>
-        <v>210</v>
+      <c r="E54" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F54">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1744</v>
       </c>
       <c r="G54">
         <v>32</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I54" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J54">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L54" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D55" s="3">
         <v>8.3951999999999999E-2</v>
       </c>
-      <c r="E55">
-        <f t="shared" si="0"/>
-        <v>214</v>
+      <c r="E55" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F55">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1776</v>
       </c>
       <c r="G55">
         <v>32</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I55" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J55">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L55" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D56" s="3">
         <v>0.14888799999999999</v>
       </c>
-      <c r="E56">
-        <f t="shared" si="0"/>
-        <v>218</v>
+      <c r="E56" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F56">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1808</v>
       </c>
       <c r="G56">
         <v>32</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I56" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J56">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L56" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D57" s="3">
         <v>0.20025299999999999</v>
       </c>
-      <c r="E57">
-        <f t="shared" si="0"/>
-        <v>222</v>
+      <c r="E57" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F57">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1840</v>
       </c>
       <c r="G57">
         <v>32</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I57" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J57">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="L57" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D58" s="3">
         <v>0.219802</v>
       </c>
-      <c r="E58">
-        <f t="shared" si="0"/>
-        <v>226</v>
+      <c r="E58" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F58">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1872</v>
       </c>
       <c r="G58">
         <v>32</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I58" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J58">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="L58" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2938,97 +3170,112 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B726021C-BBBE-4B63-A01A-6D6DD3B2E202}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="22.5" customWidth="1"/>
+    <col min="2" max="3" width="22.5" customWidth="1"/>
     <col min="5" max="6" width="14.25" customWidth="1"/>
     <col min="7" max="7" width="36.08203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>131</v>
+        <v>121</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>145</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>154</v>
+        <v>136</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>136</v>
+        <v>114</v>
+      </c>
+      <c r="C2" s="5">
+        <v>0</v>
+      </c>
+      <c r="D2" s="5">
+        <v>16</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
       <c r="G2" s="5"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>139</v>
+      <c r="A3" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="C3" s="5">
+        <f>C2+D2</f>
+        <v>16</v>
+      </c>
+      <c r="D3" s="5">
+        <v>16</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>150</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
       <c r="G3" s="5"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5" t="s">
-        <v>147</v>
+      <c r="A4" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C4" s="5">
+        <f t="shared" ref="C4:C10" si="0">C3+D3</f>
+        <v>32</v>
       </c>
       <c r="D4" s="5">
         <v>2</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>149</v>
+      <c r="E4" s="10" t="s">
+        <v>151</v>
       </c>
       <c r="F4" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" s="5"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="G4" s="5"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5" t="s">
-        <v>148</v>
+      <c r="C5" s="5">
+        <f t="shared" si="0"/>
+        <v>34</v>
       </c>
       <c r="D5" s="5">
         <v>14</v>
@@ -3037,54 +3284,65 @@
         <v>0</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>150</v>
+        <v>133</v>
       </c>
       <c r="G5" s="5" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C6" s="5">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+      <c r="D6" s="5">
+        <v>16</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="5">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+      <c r="D7" s="5">
+        <v>16</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>155</v>
-      </c>
       <c r="F7" s="5" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
       <c r="G7" s="5"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="C8" s="5">
+        <f t="shared" si="0"/>
+        <v>80</v>
       </c>
       <c r="D8" s="5">
         <v>32</v>
@@ -3093,17 +3351,42 @@
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
     </row>
-    <row r="9" spans="1:7" ht="28" x14ac:dyDescent="0.3">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="D9" s="5"/>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="C9" s="5">
+        <f t="shared" si="0"/>
+        <v>112</v>
+      </c>
+      <c r="D9" s="5">
+        <v>32</v>
+      </c>
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
-      <c r="G9" s="5" t="s">
-        <v>146</v>
+      <c r="G9" s="5"/>
+    </row>
+    <row r="10" spans="1:7" ht="28" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="C10" s="5">
+        <f t="shared" si="0"/>
+        <v>144</v>
+      </c>
+      <c r="D10" s="5">
+        <v>16</v>
+      </c>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>